<commit_message>
update extraction and recoding scripts
</commit_message>
<xml_diff>
--- a/extraction_and_recoding_new/parameters/parameters_changed.xlsx
+++ b/extraction_and_recoding_new/parameters/parameters_changed.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="959" uniqueCount="959">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="951" uniqueCount="951">
   <si>
     <t xml:space="preserve">Field</t>
   </si>
@@ -701,7 +701,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=2020</t>
   </si>
   <si>
-    <t xml:space="preserve">loneliness</t>
+    <t xml:space="preserve">mh_loneliness</t>
   </si>
   <si>
     <t xml:space="preserve">Able to confide</t>
@@ -716,7 +716,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=2110</t>
   </si>
   <si>
-    <t xml:space="preserve">social_support_confide</t>
+    <t xml:space="preserve">mh_social_support_confide</t>
   </si>
   <si>
     <t xml:space="preserve">Had major operations</t>
@@ -731,7 +731,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=2415</t>
   </si>
   <si>
-    <t xml:space="preserve">hx_major_surgery_yn</t>
+    <t xml:space="preserve">sur_major_surgery</t>
   </si>
   <si>
     <t xml:space="preserve">Diabetes diagnosed by doctor</t>
@@ -746,7 +746,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=2443</t>
   </si>
   <si>
-    <t xml:space="preserve">dx_diabetes_doc_yn</t>
+    <t xml:space="preserve">dis_diabetes_doc_yn</t>
   </si>
   <si>
     <t xml:space="preserve">Cancer diagnosed by doctor</t>
@@ -758,7 +758,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=2453</t>
   </si>
   <si>
-    <t xml:space="preserve">dx_cancer_doc_yn</t>
+    <t xml:space="preserve">dis_cancer_doc_yn</t>
   </si>
   <si>
     <t xml:space="preserve">Age high blood pressure diagnosed</t>
@@ -770,7 +770,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=2966</t>
   </si>
   <si>
-    <t xml:space="preserve">age_dx_htn</t>
+    <t xml:space="preserve">dis_age_highbp</t>
   </si>
   <si>
     <t xml:space="preserve">Age high blood pressure diagnosed (years)</t>
@@ -785,7 +785,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=2976</t>
   </si>
   <si>
-    <t xml:space="preserve">age_dx_diabetes</t>
+    <t xml:space="preserve">dis_age_diabetes</t>
   </si>
   <si>
     <t xml:space="preserve">Age diabetes diagnosed (years)</t>
@@ -884,7 +884,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=3894</t>
   </si>
   <si>
-    <t xml:space="preserve">age_dx_mi</t>
+    <t xml:space="preserve">dis_age_mi</t>
   </si>
   <si>
     <t xml:space="preserve">Age heart attack diagnosed (years)</t>
@@ -962,7 +962,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=6150</t>
   </si>
   <si>
-    <t xml:space="preserve">dx_cvd_doc_yn</t>
+    <t xml:space="preserve">dis_cvd_doc_yn</t>
   </si>
   <si>
     <t xml:space="preserve">Medication for cholesterol, blood pressure, diabetes, or take exogenous hormones</t>
@@ -1049,7 +1049,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=20126</t>
   </si>
   <si>
-    <t xml:space="preserve">BPD_MD_status</t>
+    <t xml:space="preserve">mh_BPD_MD</t>
   </si>
   <si>
     <t xml:space="preserve">Neuroticism score</t>
@@ -1061,7 +1061,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=20127</t>
   </si>
   <si>
-    <t xml:space="preserve">Neuroticism_score</t>
+    <t xml:space="preserve">mh_neuroticism</t>
   </si>
   <si>
     <t xml:space="preserve">Pack years of smoking</t>
@@ -1220,7 +1220,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=22150</t>
   </si>
   <si>
-    <t xml:space="preserve">age_copd</t>
+    <t xml:space="preserve">dis_age_copd</t>
   </si>
   <si>
     <t xml:space="preserve">Age idiopathic pulmonary fibrosis diagnosed by doctor</t>
@@ -1232,7 +1232,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=22155</t>
   </si>
   <si>
-    <t xml:space="preserve">age_pulmonary_fibrosis</t>
+    <t xml:space="preserve">dis_age_pulmonary_fibrosis</t>
   </si>
   <si>
     <t xml:space="preserve">Average heart rate</t>
@@ -1274,7 +1274,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=23099</t>
   </si>
   <si>
-    <t xml:space="preserve">body_fat_pct </t>
+    <t xml:space="preserve">body_fat_pct</t>
   </si>
   <si>
     <t xml:space="preserve">Body fat percentage (percent)</t>
@@ -2438,7 +2438,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=40005</t>
   </si>
   <si>
-    <t xml:space="preserve">date_of_cancer</t>
+    <t xml:space="preserve">dis_date_of_cancer</t>
   </si>
   <si>
     <t xml:space="preserve">Histology of cancer tumour</t>
@@ -2450,7 +2450,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=40011</t>
   </si>
   <si>
-    <t xml:space="preserve">history_cancer_tumour</t>
+    <t xml:space="preserve">dis_history_cancer_tumour</t>
   </si>
   <si>
     <t xml:space="preserve">Saturated fat</t>
@@ -2468,7 +2468,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=100006</t>
   </si>
   <si>
-    <t xml:space="preserve">saturated _fat</t>
+    <t xml:space="preserve">saturated_fat</t>
   </si>
   <si>
     <t xml:space="preserve">Saturated fat (g)</t>
@@ -2537,7 +2537,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=130200</t>
   </si>
   <si>
-    <t xml:space="preserve">chronic_hepatitis</t>
+    <t xml:space="preserve">dis_chronic_hepatitis</t>
   </si>
   <si>
     <t xml:space="preserve">Date E10 first reported (insulin-dependent diabetes mellitus)</t>
@@ -2552,7 +2552,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=130706</t>
   </si>
   <si>
-    <t xml:space="preserve">dt_e10_first</t>
+    <t xml:space="preserve">dis_insulin_dep_diabetes</t>
   </si>
   <si>
     <t xml:space="preserve">Date E11 first reported (non-insulin-dependent diabetes mellitus)</t>
@@ -2564,19 +2564,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=130708</t>
   </si>
   <si>
-    <t xml:space="preserve">dt_e11_first</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date E12 first reported (malnutrition-related diabetes mellitus)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date of the first occurrence of any code mapped to 3-character ICD10 E12. The code corresponds to \"malnutrition-related diabetes mellitus\". Note that events which were apparently before birth were omitted when constructing this data field.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=130710</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dt_e12_first</t>
+    <t xml:space="preserve">dis_non_insulin_dep_diabetes</t>
   </si>
   <si>
     <t xml:space="preserve">Date F20 first reported (schizophrenia)</t>
@@ -2591,7 +2579,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=130874</t>
   </si>
   <si>
-    <t xml:space="preserve">schizophrenia</t>
+    <t xml:space="preserve">dis_schizophrenia</t>
   </si>
   <si>
     <t xml:space="preserve">Date F32 first reported (depressive episode)</t>
@@ -2603,7 +2591,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=130894</t>
   </si>
   <si>
-    <t xml:space="preserve">depr_single_icd</t>
+    <t xml:space="preserve">mh_depr_single_icd</t>
   </si>
   <si>
     <t xml:space="preserve">Date F33 first reported (recurrent depressive disorder)</t>
@@ -2615,7 +2603,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=130896</t>
   </si>
   <si>
-    <t xml:space="preserve">depr_recurrent_icd</t>
+    <t xml:space="preserve">mh_depr_recurrent_icd</t>
   </si>
   <si>
     <t xml:space="preserve">Date F40 first reported (phobic anxiety disorders)</t>
@@ -2627,7 +2615,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=130904</t>
   </si>
   <si>
-    <t xml:space="preserve">anxiety_phobic_icd</t>
+    <t xml:space="preserve">mh_anxiety_phobic_icd</t>
   </si>
   <si>
     <t xml:space="preserve">Date F41 first reported (other anxiety disorders)</t>
@@ -2639,7 +2627,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=130906</t>
   </si>
   <si>
-    <t xml:space="preserve">anxiety_general_icd</t>
+    <t xml:space="preserve">mh_anxiety_general_icd</t>
   </si>
   <si>
     <t xml:space="preserve">Date G20 first reported (parkinson's disease)</t>
@@ -2654,7 +2642,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131022</t>
   </si>
   <si>
-    <t xml:space="preserve">parkinsons_disease</t>
+    <t xml:space="preserve">dis_parkinsons_disease</t>
   </si>
   <si>
     <t xml:space="preserve">Date G30 first reported (alzheimer's disease)</t>
@@ -2666,7 +2654,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131036</t>
   </si>
   <si>
-    <t xml:space="preserve">alzheimers_disease</t>
+    <t xml:space="preserve">dis_alzheimers_disease</t>
   </si>
   <si>
     <t xml:space="preserve">Date G35 first reported (multiple sclerosis)</t>
@@ -2678,7 +2666,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131042</t>
   </si>
   <si>
-    <t xml:space="preserve">multiple_sclerosis</t>
+    <t xml:space="preserve">dis_multiple_sclerosis</t>
   </si>
   <si>
     <t xml:space="preserve">Date G43 first reported (migraine)</t>
@@ -2690,7 +2678,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131052</t>
   </si>
   <si>
-    <t xml:space="preserve">migraine</t>
+    <t xml:space="preserve">dis_migraine</t>
   </si>
   <si>
     <t xml:space="preserve">Date G44 first reported (other headache syndromes)</t>
@@ -2702,7 +2690,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131054</t>
   </si>
   <si>
-    <t xml:space="preserve">other_headaches</t>
+    <t xml:space="preserve">dis_other_headaches</t>
   </si>
   <si>
     <t xml:space="preserve">Date G47 first reported (sleep disorders)</t>
@@ -2714,7 +2702,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131060</t>
   </si>
   <si>
-    <t xml:space="preserve">sleep_disorders</t>
+    <t xml:space="preserve">dis_sleep_disorders</t>
   </si>
   <si>
     <t xml:space="preserve">Date I10 first reported (essential (primary) hypertension)</t>
@@ -2729,19 +2717,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131286</t>
   </si>
   <si>
-    <t xml:space="preserve">dt_l10_first</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source of report of I10 (essential (primary) hypertension)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source of the first code mapped to 3-character ICD10 I10, and whether this code occurs in other source(s) with the same or a later event date. The code corresponds to \"essential (primary) hypertension\". See Resource 593 for details of how the first source was assigned.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131287</t>
-  </si>
-  <si>
-    <t xml:space="preserve">src_l10_first</t>
+    <t xml:space="preserve">dis_dt_l10_first</t>
   </si>
   <si>
     <t xml:space="preserve">Date I12 first reported (hypertensive renal disease)</t>
@@ -2753,7 +2729,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131290</t>
   </si>
   <si>
-    <t xml:space="preserve">hypertensive_renal_disease</t>
+    <t xml:space="preserve">dis_hypertensive_renal_disease</t>
   </si>
   <si>
     <t xml:space="preserve">Date I13 first reported (hypertensive heart and renal disease)</t>
@@ -2765,7 +2741,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131292</t>
   </si>
   <si>
-    <t xml:space="preserve">hypertensive_heart_renal_disease</t>
+    <t xml:space="preserve">dis_hypertensive_heart_renal_disease</t>
   </si>
   <si>
     <t xml:space="preserve">Date J45 first reported (asthma)</t>
@@ -2780,7 +2756,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131494</t>
   </si>
   <si>
-    <t xml:space="preserve">asthma</t>
+    <t xml:space="preserve">dis_asthma</t>
   </si>
   <si>
     <t xml:space="preserve">Date K50 first reported (crohn's disease [regional enteritis])</t>
@@ -2795,7 +2771,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131626</t>
   </si>
   <si>
-    <t xml:space="preserve">crohns_disease</t>
+    <t xml:space="preserve">dis_crohns_disease</t>
   </si>
   <si>
     <t xml:space="preserve">Date K51 first reported (ulcerative colitis)</t>
@@ -2807,7 +2783,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131628</t>
   </si>
   <si>
-    <t xml:space="preserve">ulcerative_colitis</t>
+    <t xml:space="preserve">dis_ulcerative_colitis</t>
   </si>
   <si>
     <t xml:space="preserve">Date K70 first reported (alcoholic liver disease)</t>
@@ -2819,7 +2795,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131658</t>
   </si>
   <si>
-    <t xml:space="preserve">alcoholic _liver_disease</t>
+    <t xml:space="preserve">dis_alcoholic_liver_disease</t>
   </si>
   <si>
     <t xml:space="preserve">Date K74 first reported (fibrosis and cirrhosis of liver)</t>
@@ -2831,7 +2807,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131666</t>
   </si>
   <si>
-    <t xml:space="preserve">liver_fibrosis_and_cirrhosis</t>
+    <t xml:space="preserve">dis_liver_fibrosis_and_cirrhosis</t>
   </si>
   <si>
     <t xml:space="preserve">Date L40 first reported (psoriasis)</t>
@@ -2846,7 +2822,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131742</t>
   </si>
   <si>
-    <t xml:space="preserve">psoriasis</t>
+    <t xml:space="preserve">dis_psoriasis</t>
   </si>
   <si>
     <t xml:space="preserve">Date L93 first reported (lupus erythematosus)</t>
@@ -2858,7 +2834,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131828</t>
   </si>
   <si>
-    <t xml:space="preserve">lupus</t>
+    <t xml:space="preserve">dis_lupus</t>
   </si>
   <si>
     <t xml:space="preserve">Date M05 first reported (seropositive rheumatoid arthritis)</t>
@@ -2873,7 +2849,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=131848</t>
   </si>
   <si>
-    <t xml:space="preserve">rheumatoid_arthritis</t>
+    <t xml:space="preserve">dis_rheumatoid_arthritis</t>
   </si>
   <si>
     <t xml:space="preserve">Date N18 first reported (chronic renal failure)</t>
@@ -2888,7 +2864,7 @@
     <t xml:space="preserve">http://biobank.ndph.ox.ac.uk/ukb/field.cgi?id=132032</t>
   </si>
   <si>
-    <t xml:space="preserve">chronic_renal_failure</t>
+    <t xml:space="preserve">dis_chronic_renal_failure</t>
   </si>
 </sst>
 </file>
@@ -11247,7 +11223,7 @@
         <v>851</v>
       </c>
       <c r="B160" t="n">
-        <v>8</v>
+        <v>1461</v>
       </c>
       <c r="C160" t="s">
         <v>852</v>
@@ -11257,13 +11233,13 @@
         <v>19</v>
       </c>
       <c r="F160" t="s">
-        <v>844</v>
+        <v>853</v>
       </c>
       <c r="G160" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="H160" t="n">
-        <v>130710</v>
+        <v>130874</v>
       </c>
       <c r="I160" t="s">
         <v>27</v>
@@ -11272,7 +11248,7 @@
         <v>819</v>
       </c>
       <c r="K160" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="L160" t="s">
         <v>851</v>
@@ -11293,26 +11269,26 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="B161" t="n">
-        <v>1461</v>
+        <v>63043</v>
       </c>
       <c r="C161" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="D161"/>
       <c r="E161" t="s">
         <v>19</v>
       </c>
       <c r="F161" t="s">
-        <v>857</v>
+        <v>853</v>
       </c>
       <c r="G161" t="s">
         <v>858</v>
       </c>
       <c r="H161" t="n">
-        <v>130874</v>
+        <v>130894</v>
       </c>
       <c r="I161" t="s">
         <v>27</v>
@@ -11324,14 +11300,14 @@
         <v>859</v>
       </c>
       <c r="L161" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="M161"/>
       <c r="N161" t="s">
         <v>19</v>
       </c>
       <c r="O161" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="P161" t="s">
         <v>19</v>
@@ -11345,7 +11321,7 @@
         <v>860</v>
       </c>
       <c r="B162" t="n">
-        <v>63043</v>
+        <v>3966</v>
       </c>
       <c r="C162" t="s">
         <v>861</v>
@@ -11355,13 +11331,13 @@
         <v>19</v>
       </c>
       <c r="F162" t="s">
-        <v>857</v>
+        <v>853</v>
       </c>
       <c r="G162" t="s">
         <v>862</v>
       </c>
       <c r="H162" t="n">
-        <v>130894</v>
+        <v>130896</v>
       </c>
       <c r="I162" t="s">
         <v>27</v>
@@ -11394,7 +11370,7 @@
         <v>864</v>
       </c>
       <c r="B163" t="n">
-        <v>3966</v>
+        <v>4499</v>
       </c>
       <c r="C163" t="s">
         <v>865</v>
@@ -11404,13 +11380,13 @@
         <v>19</v>
       </c>
       <c r="F163" t="s">
-        <v>857</v>
+        <v>853</v>
       </c>
       <c r="G163" t="s">
         <v>866</v>
       </c>
       <c r="H163" t="n">
-        <v>130896</v>
+        <v>130904</v>
       </c>
       <c r="I163" t="s">
         <v>27</v>
@@ -11443,7 +11419,7 @@
         <v>868</v>
       </c>
       <c r="B164" t="n">
-        <v>4499</v>
+        <v>42018</v>
       </c>
       <c r="C164" t="s">
         <v>869</v>
@@ -11453,13 +11429,13 @@
         <v>19</v>
       </c>
       <c r="F164" t="s">
-        <v>857</v>
+        <v>853</v>
       </c>
       <c r="G164" t="s">
         <v>870</v>
       </c>
       <c r="H164" t="n">
-        <v>130904</v>
+        <v>130906</v>
       </c>
       <c r="I164" t="s">
         <v>27</v>
@@ -11492,7 +11468,7 @@
         <v>872</v>
       </c>
       <c r="B165" t="n">
-        <v>42018</v>
+        <v>4564</v>
       </c>
       <c r="C165" t="s">
         <v>873</v>
@@ -11502,13 +11478,13 @@
         <v>19</v>
       </c>
       <c r="F165" t="s">
-        <v>857</v>
+        <v>874</v>
       </c>
       <c r="G165" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="H165" t="n">
-        <v>130906</v>
+        <v>131022</v>
       </c>
       <c r="I165" t="s">
         <v>27</v>
@@ -11517,7 +11493,7 @@
         <v>819</v>
       </c>
       <c r="K165" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="L165" t="s">
         <v>872</v>
@@ -11538,26 +11514,26 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="B166" t="n">
-        <v>4564</v>
+        <v>4473</v>
       </c>
       <c r="C166" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="D166"/>
       <c r="E166" t="s">
         <v>19</v>
       </c>
       <c r="F166" t="s">
-        <v>878</v>
+        <v>874</v>
       </c>
       <c r="G166" t="s">
         <v>879</v>
       </c>
       <c r="H166" t="n">
-        <v>131022</v>
+        <v>131036</v>
       </c>
       <c r="I166" t="s">
         <v>27</v>
@@ -11569,14 +11545,14 @@
         <v>880</v>
       </c>
       <c r="L166" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="M166"/>
       <c r="N166" t="s">
         <v>19</v>
       </c>
       <c r="O166" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="P166" t="s">
         <v>19</v>
@@ -11590,7 +11566,7 @@
         <v>881</v>
       </c>
       <c r="B167" t="n">
-        <v>4473</v>
+        <v>2595</v>
       </c>
       <c r="C167" t="s">
         <v>882</v>
@@ -11600,13 +11576,13 @@
         <v>19</v>
       </c>
       <c r="F167" t="s">
-        <v>878</v>
+        <v>874</v>
       </c>
       <c r="G167" t="s">
         <v>883</v>
       </c>
       <c r="H167" t="n">
-        <v>131036</v>
+        <v>131042</v>
       </c>
       <c r="I167" t="s">
         <v>27</v>
@@ -11639,7 +11615,7 @@
         <v>885</v>
       </c>
       <c r="B168" t="n">
-        <v>2595</v>
+        <v>27402</v>
       </c>
       <c r="C168" t="s">
         <v>886</v>
@@ -11649,13 +11625,13 @@
         <v>19</v>
       </c>
       <c r="F168" t="s">
-        <v>878</v>
+        <v>874</v>
       </c>
       <c r="G168" t="s">
         <v>887</v>
       </c>
       <c r="H168" t="n">
-        <v>131042</v>
+        <v>131052</v>
       </c>
       <c r="I168" t="s">
         <v>27</v>
@@ -11688,7 +11664,7 @@
         <v>889</v>
       </c>
       <c r="B169" t="n">
-        <v>27402</v>
+        <v>6180</v>
       </c>
       <c r="C169" t="s">
         <v>890</v>
@@ -11698,13 +11674,13 @@
         <v>19</v>
       </c>
       <c r="F169" t="s">
-        <v>878</v>
+        <v>874</v>
       </c>
       <c r="G169" t="s">
         <v>891</v>
       </c>
       <c r="H169" t="n">
-        <v>131052</v>
+        <v>131054</v>
       </c>
       <c r="I169" t="s">
         <v>27</v>
@@ -11737,7 +11713,7 @@
         <v>893</v>
       </c>
       <c r="B170" t="n">
-        <v>6180</v>
+        <v>21013</v>
       </c>
       <c r="C170" t="s">
         <v>894</v>
@@ -11747,13 +11723,13 @@
         <v>19</v>
       </c>
       <c r="F170" t="s">
-        <v>878</v>
+        <v>874</v>
       </c>
       <c r="G170" t="s">
         <v>895</v>
       </c>
       <c r="H170" t="n">
-        <v>131054</v>
+        <v>131060</v>
       </c>
       <c r="I170" t="s">
         <v>27</v>
@@ -11786,7 +11762,7 @@
         <v>897</v>
       </c>
       <c r="B171" t="n">
-        <v>21013</v>
+        <v>203053</v>
       </c>
       <c r="C171" t="s">
         <v>898</v>
@@ -11796,13 +11772,13 @@
         <v>19</v>
       </c>
       <c r="F171" t="s">
-        <v>878</v>
+        <v>899</v>
       </c>
       <c r="G171" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="H171" t="n">
-        <v>131060</v>
+        <v>131286</v>
       </c>
       <c r="I171" t="s">
         <v>27</v>
@@ -11811,7 +11787,7 @@
         <v>819</v>
       </c>
       <c r="K171" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="L171" t="s">
         <v>897</v>
@@ -11832,26 +11808,26 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="B172" t="n">
-        <v>203053</v>
+        <v>2283</v>
       </c>
       <c r="C172" t="s">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="D172"/>
       <c r="E172" t="s">
         <v>19</v>
       </c>
       <c r="F172" t="s">
-        <v>903</v>
+        <v>899</v>
       </c>
       <c r="G172" t="s">
         <v>904</v>
       </c>
       <c r="H172" t="n">
-        <v>131286</v>
+        <v>131290</v>
       </c>
       <c r="I172" t="s">
         <v>27</v>
@@ -11863,14 +11839,14 @@
         <v>905</v>
       </c>
       <c r="L172" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="M172"/>
       <c r="N172" t="s">
         <v>19</v>
       </c>
       <c r="O172" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="P172" t="s">
         <v>19</v>
@@ -11884,7 +11860,7 @@
         <v>906</v>
       </c>
       <c r="B173" t="n">
-        <v>203053</v>
+        <v>199</v>
       </c>
       <c r="C173" t="s">
         <v>907</v>
@@ -11894,19 +11870,19 @@
         <v>19</v>
       </c>
       <c r="F173" t="s">
-        <v>903</v>
+        <v>899</v>
       </c>
       <c r="G173" t="s">
         <v>908</v>
       </c>
       <c r="H173" t="n">
-        <v>131287</v>
+        <v>131292</v>
       </c>
       <c r="I173" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="J173" t="n">
-        <v>2171</v>
+        <v>819</v>
       </c>
       <c r="K173" t="s">
         <v>909</v>
@@ -11933,7 +11909,7 @@
         <v>910</v>
       </c>
       <c r="B174" t="n">
-        <v>2283</v>
+        <v>74348</v>
       </c>
       <c r="C174" t="s">
         <v>911</v>
@@ -11943,13 +11919,13 @@
         <v>19</v>
       </c>
       <c r="F174" t="s">
-        <v>903</v>
+        <v>912</v>
       </c>
       <c r="G174" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="H174" t="n">
-        <v>131290</v>
+        <v>131494</v>
       </c>
       <c r="I174" t="s">
         <v>27</v>
@@ -11958,7 +11934,7 @@
         <v>819</v>
       </c>
       <c r="K174" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="L174" t="s">
         <v>910</v>
@@ -11979,26 +11955,26 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="B175" t="n">
-        <v>199</v>
+        <v>3502</v>
       </c>
       <c r="C175" t="s">
-        <v>915</v>
+        <v>916</v>
       </c>
       <c r="D175"/>
       <c r="E175" t="s">
         <v>19</v>
       </c>
       <c r="F175" t="s">
-        <v>903</v>
+        <v>917</v>
       </c>
       <c r="G175" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="H175" t="n">
-        <v>131292</v>
+        <v>131626</v>
       </c>
       <c r="I175" t="s">
         <v>27</v>
@@ -12007,17 +11983,17 @@
         <v>819</v>
       </c>
       <c r="K175" t="s">
-        <v>917</v>
+        <v>919</v>
       </c>
       <c r="L175" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="M175"/>
       <c r="N175" t="s">
         <v>19</v>
       </c>
       <c r="O175" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
       <c r="P175" t="s">
         <v>19</v>
@@ -12028,26 +12004,26 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>918</v>
+        <v>920</v>
       </c>
       <c r="B176" t="n">
-        <v>74348</v>
+        <v>6698</v>
       </c>
       <c r="C176" t="s">
-        <v>919</v>
+        <v>921</v>
       </c>
       <c r="D176"/>
       <c r="E176" t="s">
         <v>19</v>
       </c>
       <c r="F176" t="s">
-        <v>920</v>
+        <v>917</v>
       </c>
       <c r="G176" t="s">
-        <v>921</v>
+        <v>922</v>
       </c>
       <c r="H176" t="n">
-        <v>131494</v>
+        <v>131628</v>
       </c>
       <c r="I176" t="s">
         <v>27</v>
@@ -12056,17 +12032,17 @@
         <v>819</v>
       </c>
       <c r="K176" t="s">
-        <v>922</v>
+        <v>923</v>
       </c>
       <c r="L176" t="s">
-        <v>918</v>
+        <v>920</v>
       </c>
       <c r="M176"/>
       <c r="N176" t="s">
         <v>19</v>
       </c>
       <c r="O176" t="s">
-        <v>918</v>
+        <v>920</v>
       </c>
       <c r="P176" t="s">
         <v>19</v>
@@ -12077,26 +12053,26 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
       <c r="B177" t="n">
-        <v>3502</v>
+        <v>2441</v>
       </c>
       <c r="C177" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
       <c r="D177"/>
       <c r="E177" t="s">
         <v>19</v>
       </c>
       <c r="F177" t="s">
-        <v>925</v>
+        <v>917</v>
       </c>
       <c r="G177" t="s">
         <v>926</v>
       </c>
       <c r="H177" t="n">
-        <v>131626</v>
+        <v>131658</v>
       </c>
       <c r="I177" t="s">
         <v>27</v>
@@ -12108,14 +12084,14 @@
         <v>927</v>
       </c>
       <c r="L177" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
       <c r="M177"/>
       <c r="N177" t="s">
         <v>19</v>
       </c>
       <c r="O177" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
       <c r="P177" t="s">
         <v>19</v>
@@ -12129,7 +12105,7 @@
         <v>928</v>
       </c>
       <c r="B178" t="n">
-        <v>6698</v>
+        <v>3104</v>
       </c>
       <c r="C178" t="s">
         <v>929</v>
@@ -12139,13 +12115,13 @@
         <v>19</v>
       </c>
       <c r="F178" t="s">
-        <v>925</v>
+        <v>917</v>
       </c>
       <c r="G178" t="s">
         <v>930</v>
       </c>
       <c r="H178" t="n">
-        <v>131628</v>
+        <v>131666</v>
       </c>
       <c r="I178" t="s">
         <v>27</v>
@@ -12178,7 +12154,7 @@
         <v>932</v>
       </c>
       <c r="B179" t="n">
-        <v>2441</v>
+        <v>15928</v>
       </c>
       <c r="C179" t="s">
         <v>933</v>
@@ -12188,13 +12164,13 @@
         <v>19</v>
       </c>
       <c r="F179" t="s">
-        <v>925</v>
+        <v>934</v>
       </c>
       <c r="G179" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
       <c r="H179" t="n">
-        <v>131658</v>
+        <v>131742</v>
       </c>
       <c r="I179" t="s">
         <v>27</v>
@@ -12203,7 +12179,7 @@
         <v>819</v>
       </c>
       <c r="K179" t="s">
-        <v>935</v>
+        <v>936</v>
       </c>
       <c r="L179" t="s">
         <v>932</v>
@@ -12224,26 +12200,26 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="B180" t="n">
-        <v>3104</v>
+        <v>552</v>
       </c>
       <c r="C180" t="s">
-        <v>937</v>
+        <v>938</v>
       </c>
       <c r="D180"/>
       <c r="E180" t="s">
         <v>19</v>
       </c>
       <c r="F180" t="s">
-        <v>925</v>
+        <v>934</v>
       </c>
       <c r="G180" t="s">
-        <v>938</v>
+        <v>939</v>
       </c>
       <c r="H180" t="n">
-        <v>131666</v>
+        <v>131828</v>
       </c>
       <c r="I180" t="s">
         <v>27</v>
@@ -12252,17 +12228,17 @@
         <v>819</v>
       </c>
       <c r="K180" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="L180" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="M180"/>
       <c r="N180" t="s">
         <v>19</v>
       </c>
       <c r="O180" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="P180" t="s">
         <v>19</v>
@@ -12273,26 +12249,26 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="B181" t="n">
-        <v>15928</v>
+        <v>1534</v>
       </c>
       <c r="C181" t="s">
-        <v>941</v>
+        <v>942</v>
       </c>
       <c r="D181"/>
       <c r="E181" t="s">
         <v>19</v>
       </c>
       <c r="F181" t="s">
-        <v>942</v>
+        <v>943</v>
       </c>
       <c r="G181" t="s">
-        <v>943</v>
+        <v>944</v>
       </c>
       <c r="H181" t="n">
-        <v>131742</v>
+        <v>131848</v>
       </c>
       <c r="I181" t="s">
         <v>27</v>
@@ -12301,17 +12277,17 @@
         <v>819</v>
       </c>
       <c r="K181" t="s">
-        <v>944</v>
+        <v>945</v>
       </c>
       <c r="L181" t="s">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="M181"/>
       <c r="N181" t="s">
         <v>19</v>
       </c>
       <c r="O181" t="s">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="P181" t="s">
         <v>19</v>
@@ -12322,26 +12298,26 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="B182" t="n">
-        <v>552</v>
+        <v>31231</v>
       </c>
       <c r="C182" t="s">
-        <v>946</v>
+        <v>947</v>
       </c>
       <c r="D182"/>
       <c r="E182" t="s">
         <v>19</v>
       </c>
       <c r="F182" t="s">
-        <v>942</v>
+        <v>948</v>
       </c>
       <c r="G182" t="s">
-        <v>947</v>
+        <v>949</v>
       </c>
       <c r="H182" t="n">
-        <v>131828</v>
+        <v>132032</v>
       </c>
       <c r="I182" t="s">
         <v>27</v>
@@ -12350,120 +12326,22 @@
         <v>819</v>
       </c>
       <c r="K182" t="s">
-        <v>948</v>
+        <v>950</v>
       </c>
       <c r="L182" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="M182"/>
       <c r="N182" t="s">
         <v>19</v>
       </c>
       <c r="O182" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="P182" t="s">
         <v>19</v>
       </c>
       <c r="Q182" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="s">
-        <v>949</v>
-      </c>
-      <c r="B183" t="n">
-        <v>1534</v>
-      </c>
-      <c r="C183" t="s">
-        <v>950</v>
-      </c>
-      <c r="D183"/>
-      <c r="E183" t="s">
-        <v>19</v>
-      </c>
-      <c r="F183" t="s">
-        <v>951</v>
-      </c>
-      <c r="G183" t="s">
-        <v>952</v>
-      </c>
-      <c r="H183" t="n">
-        <v>131848</v>
-      </c>
-      <c r="I183" t="s">
-        <v>27</v>
-      </c>
-      <c r="J183" t="n">
-        <v>819</v>
-      </c>
-      <c r="K183" t="s">
-        <v>953</v>
-      </c>
-      <c r="L183" t="s">
-        <v>949</v>
-      </c>
-      <c r="M183"/>
-      <c r="N183" t="s">
-        <v>19</v>
-      </c>
-      <c r="O183" t="s">
-        <v>949</v>
-      </c>
-      <c r="P183" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q183" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="s">
-        <v>954</v>
-      </c>
-      <c r="B184" t="n">
-        <v>31231</v>
-      </c>
-      <c r="C184" t="s">
-        <v>955</v>
-      </c>
-      <c r="D184"/>
-      <c r="E184" t="s">
-        <v>19</v>
-      </c>
-      <c r="F184" t="s">
-        <v>956</v>
-      </c>
-      <c r="G184" t="s">
-        <v>957</v>
-      </c>
-      <c r="H184" t="n">
-        <v>132032</v>
-      </c>
-      <c r="I184" t="s">
-        <v>27</v>
-      </c>
-      <c r="J184" t="n">
-        <v>819</v>
-      </c>
-      <c r="K184" t="s">
-        <v>958</v>
-      </c>
-      <c r="L184" t="s">
-        <v>954</v>
-      </c>
-      <c r="M184"/>
-      <c r="N184" t="s">
-        <v>19</v>
-      </c>
-      <c r="O184" t="s">
-        <v>954</v>
-      </c>
-      <c r="P184" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q184" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>